<commit_message>
fix: move .Meta to first sheet position in Config_Reference
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/Config_Reference.xlsx
+++ b/test/fixtures/Config_Reference.xlsx
@@ -7,13 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Constants" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Environments" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Features" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Assets" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Connections" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name=".Meta" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name=".Meta" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Settings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Constants" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Environments" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Features" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Assets" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Connections" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name=".Notes" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
@@ -430,130 +430,66 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Key</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Value</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Description</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>OrchestratorQueueName</t>
+          <t>Author</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>everything_input_queue</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>string — Orchestrator input queue name.</t>
+          <t>ConFigTree</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MaxItemsPerRun</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>100</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>int — Maximum items to process per run.</t>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Threshold</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>3.14</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>double — Processing threshold.</t>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Documentation master fixture — all types, all sheet kinds.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IsEnabled</t>
-        </is>
-      </c>
-      <c r="B5" t="b">
-        <v>1</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>bool — Master feature toggle.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CutoffDate</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>46022</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>DateOnly — Last valid processing date.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>ScheduledAt</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>45823.39583333334</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>DateTime — Next scheduled run.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>DailyRunTime</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>TimeOnly — Daily start time.</t>
+          <t>GeneratedBy</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>generate_fixtures.py</t>
         </is>
       </c>
     </row>
@@ -568,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -591,120 +527,107 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MaxRetryNumber</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0</v>
+          <t>OrchestratorQueueName</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>everything_input_queue</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>int — Must be 0 when using Orchestrator queues.</t>
+          <t>string — Orchestrator input queue name.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MaxConsecutiveSystemExceptions</t>
+          <t>MaxItemsPerRun</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>int — Stop job after this many consecutive errors.</t>
+          <t>int — Maximum items to process per run.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pi</t>
+          <t>Threshold</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.14159</v>
+        <v>3.14</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>double — Mathematical constant.</t>
+          <t>double — Processing threshold.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>StrictMode</t>
+          <t>IsEnabled</t>
         </is>
       </c>
       <c r="B5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>bool — Disable for permissive validation.</t>
+          <t>bool — Master feature toggle.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ExpiresOn</t>
+          <t>CutoffDate</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>46023</v>
+        <v>46022</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DateOnly — Config expiry date.</t>
+          <t>DateOnly — Last valid processing date.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CreatedAt</t>
+          <t>ScheduledAt</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>45352.5</v>
+        <v>45823.39583333334</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DateTime — Config creation timestamp.</t>
+          <t>DateTime — Next scheduled run.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>WindowOpen</t>
+          <t>DailyRunTime</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>0.375</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>TimeOnly — Processing window start.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>WindowClose</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>0.7291666666666666</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>TimeOnly — Processing window end.</t>
+          <t>TimeOnly — Daily start time.</t>
         </is>
       </c>
     </row>
@@ -719,7 +642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -742,64 +665,120 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BaseUrl</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://uat.example.com</t>
-        </is>
+          <t>MaxRetryNumber</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>string — REST API base URL.</t>
+          <t>int — Must be 0 when using Orchestrator queues.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Environment</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>UAT</t>
-        </is>
+          <t>MaxConsecutiveSystemExceptions</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>string — Deployment environment name.</t>
+          <t>int — Stop job after this many consecutive errors.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Timeout</t>
+          <t>Pi</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>30</v>
+        <v>3.14159</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>int — HTTP request timeout in seconds.</t>
+          <t>double — Mathematical constant.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RetryDelay</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2.5</v>
+          <t>StrictMode</t>
+        </is>
+      </c>
+      <c r="B5" t="b">
+        <v>0</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>double — Delay between retries in seconds.</t>
+          <t>bool — Disable for permissive validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ExpiresOn</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>46023</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DateOnly — Config expiry date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CreatedAt</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>45352.5</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DateTime — Config creation timestamp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>WindowOpen</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TimeOnly — Processing window start.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>WindowClose</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>0.7291666666666666</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TimeOnly — Processing window end.</t>
         </is>
       </c>
     </row>
@@ -837,62 +816,64 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EnableNotifications</t>
-        </is>
-      </c>
-      <c r="B2" t="b">
-        <v>1</v>
+          <t>BaseUrl</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://uat.example.com</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>bool — Send email on job completion.</t>
+          <t>string — REST API base URL.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EnableDryRun</t>
-        </is>
-      </c>
-      <c r="B3" t="b">
-        <v>0</v>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>UAT</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>bool — Skip writes when true.</t>
+          <t>string — Deployment environment name.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MaxParallelJobs</t>
+          <t>Timeout</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>int — Parallel job slot limit.</t>
+          <t>int — HTTP request timeout in seconds.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FeatureLabel</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>beta</t>
-        </is>
+          <t>RetryDelay</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2.5</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>string — Deployment stage label.</t>
+          <t>double — Delay between retries in seconds.</t>
         </is>
       </c>
     </row>
@@ -907,7 +888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -918,125 +899,74 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Asset</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>OrchestratorAssetFolder</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
           <t>Description</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>ValueType</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>QueueName</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>cfgtree_queue_name</t>
-        </is>
+          <t>EnableNotifications</t>
+        </is>
+      </c>
+      <c r="B2" t="b">
+        <v>1</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CPMForge</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Input queue name.</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>string</t>
+          <t>bool — Send email on job completion.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MaxItemsPerRun</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>cfgtree_max_items_per_run</t>
-        </is>
+          <t>EnableDryRun</t>
+        </is>
+      </c>
+      <c r="B3" t="b">
+        <v>0</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CPMForge</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Maximum items to process.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>int</t>
+          <t>bool — Skip writes when true.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>StrictMode</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>cfgtree_strict_mode</t>
-        </is>
+          <t>MaxParallelJobs</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CPMForge</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Strict processing toggle.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>bool</t>
+          <t>int — Parallel job slot limit.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GenericValue</t>
+          <t>FeatureLabel</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>cfgtree_generic_value</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CPMForge</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Untyped fallback asset.</t>
+          <t>string — Deployment stage label.</t>
         </is>
       </c>
     </row>
@@ -1051,7 +981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1084,12 +1014,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ApiEndpoint</t>
+          <t>QueueName</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>cfgtree_api_endpoint</t>
+          <t>cfgtree_queue_name</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1099,7 +1029,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>REST API endpoint URL.</t>
+          <t>Input queue name.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1111,12 +1041,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BaseUrl</t>
+          <t>MaxItemsPerRun</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>cfgtree_base_url</t>
+          <t>cfgtree_max_items_per_run</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1126,24 +1056,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Service base URL.</t>
+          <t>Maximum items to process.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>OrchestratorFolder</t>
+          <t>StrictMode</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>cfgtree_orch_folder</t>
+          <t>cfgtree_strict_mode</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1153,12 +1083,34 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Orchestrator folder path.</t>
+          <t>Strict processing toggle.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>bool</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GenericValue</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>cfgtree_generic_value</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CPMForge</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Untyped fallback asset.</t>
         </is>
       </c>
     </row>
@@ -1173,66 +1125,114 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Key</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Asset</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>OrchestratorAssetFolder</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ValueType</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Author</t>
+          <t>ApiEndpoint</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ConFigTree</t>
+          <t>cfgtree_api_endpoint</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CPMForge</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>REST API endpoint URL.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>string</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>BaseUrl</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1.0.0</t>
+          <t>cfgtree_base_url</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CPMForge</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Service base URL.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>string</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>OrchestratorFolder</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Documentation master fixture — all types, all sheet kinds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>GeneratedBy</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>generate_fixtures.py</t>
+          <t>cfgtree_orch_folder</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CPMForge</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Orchestrator folder path.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>string</t>
         </is>
       </c>
     </row>

</xml_diff>